<commit_message>
feat(courses): complete summaries results ratings and course reports
</commit_message>
<xml_diff>
--- a/docs/ke-hoach/SWP391_TaskSheet_Sprint4.xlsx
+++ b/docs/ke-hoach/SWP391_TaskSheet_Sprint4.xlsx
@@ -1290,7 +1290,7 @@
       </c>
       <c r="K16" s="6" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Review</t>
         </is>
       </c>
       <c r="L16" s="7" t="inlineStr">
@@ -1352,7 +1352,7 @@
       </c>
       <c r="K17" s="6" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Review</t>
         </is>
       </c>
       <c r="L17" s="7" t="inlineStr">
@@ -1476,7 +1476,7 @@
       </c>
       <c r="K19" s="6" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Review</t>
         </is>
       </c>
       <c r="L19" s="7" t="inlineStr">
@@ -1600,7 +1600,7 @@
       </c>
       <c r="K21" s="6" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Review</t>
         </is>
       </c>
       <c r="L21" s="7" t="inlineStr">
@@ -1724,7 +1724,7 @@
       </c>
       <c r="K23" s="6" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Review</t>
         </is>
       </c>
       <c r="L23" s="7" t="inlineStr">
@@ -1848,7 +1848,7 @@
       </c>
       <c r="K25" s="6" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Review</t>
         </is>
       </c>
       <c r="L25" s="7" t="inlineStr">

</xml_diff>

<commit_message>
feat(reports): group revenue and member trends with reconciled breakdowns
</commit_message>
<xml_diff>
--- a/docs/ke-hoach/SWP391_TaskSheet_Sprint4.xlsx
+++ b/docs/ke-hoach/SWP391_TaskSheet_Sprint4.xlsx
@@ -1972,7 +1972,7 @@
       </c>
       <c r="K27" s="6" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Review</t>
         </is>
       </c>
       <c r="L27" s="7" t="inlineStr">
@@ -2096,7 +2096,7 @@
       </c>
       <c r="K29" s="6" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Review</t>
         </is>
       </c>
       <c r="L29" s="7" t="inlineStr">
@@ -2220,7 +2220,7 @@
       </c>
       <c r="K31" s="6" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Review</t>
         </is>
       </c>
       <c r="L31" s="7" t="inlineStr">
@@ -2344,7 +2344,7 @@
       </c>
       <c r="K33" s="6" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Review</t>
         </is>
       </c>
       <c r="L33" s="7" t="inlineStr">

</xml_diff>

<commit_message>
feat(reports): add interactive period comparison and member dashboards
</commit_message>
<xml_diff>
--- a/docs/ke-hoach/SWP391_TaskSheet_Sprint4.xlsx
+++ b/docs/ke-hoach/SWP391_TaskSheet_Sprint4.xlsx
@@ -2034,7 +2034,7 @@
       </c>
       <c r="K28" s="6" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Review</t>
         </is>
       </c>
       <c r="L28" s="7" t="inlineStr">
@@ -2158,7 +2158,7 @@
       </c>
       <c r="K30" s="6" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Review</t>
         </is>
       </c>
       <c r="L30" s="7" t="inlineStr">
@@ -2282,7 +2282,7 @@
       </c>
       <c r="K32" s="6" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Review</t>
         </is>
       </c>
       <c r="L32" s="7" t="inlineStr">

</xml_diff>

<commit_message>
docs(sprint4): record requirements test evidence and final demo handover
</commit_message>
<xml_diff>
--- a/docs/ke-hoach/SWP391_TaskSheet_Sprint4.xlsx
+++ b/docs/ke-hoach/SWP391_TaskSheet_Sprint4.xlsx
@@ -2592,7 +2592,7 @@
       </c>
       <c r="K37" s="6" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Review</t>
         </is>
       </c>
       <c r="L37" s="7" t="inlineStr">
@@ -2716,12 +2716,12 @@
       </c>
       <c r="K39" s="6" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="L39" s="7" t="inlineStr">
         <is>
-          <t>#126. Khoá code 16/11. · Chuyển từ Nhanh sang Bảo theo phân công 29/10/2026.</t>
+          <t>#126. Khoá code 16/11. · Chuyển từ Nhanh sang Bảo theo phân công 29/10/2026. · Đã chuẩn bị kịch bản và test tự động; chờ diễn tập trực tiếp cả nhóm sau tích hợp Khôi/Khải.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(sprint4): deliver Khai test cases and verified handover (S4-31)
</commit_message>
<xml_diff>
--- a/docs/ke-hoach/SWP391_TaskSheet_Sprint4.xlsx
+++ b/docs/ke-hoach/SWP391_TaskSheet_Sprint4.xlsx
@@ -291,289 +291,289 @@
     <t>sprint-4/fe-khai</t>
   </si>
   <si>
+    <t>Màn S37, làm theo contract trước, giả lập dữ liệu nếu BE chưa xong · Khải hoàn thiện 29/10/2026 trên sprint-4/fe-khai; bàn giao docs/handover/sprint-4-fe-khai.md. Đã xác minh 238 BE, 160 FE và đủ 86 E2E desktop sau chạy lại; 15 test case bổ sung, chờ leader review.</t>
+  </si>
+  <si>
+    <t>S4-14</t>
+  </si>
+  <si>
+    <t>BE – Công bố / mở lại tổng kết: HLV bấm Công bố → khoá bản tổng kết, gửi thông báo in-app + email cho từng học viên. Sau khi công bố chỉ quản lý được mở lại (nhập lý do), HLV sửa và công bố lại thì hội viên nhận thông báo cập nhật.</t>
+  </si>
+  <si>
+    <t>BR-S4-09: chỉ công bố khi mọi học viên đã có kết quả. Công bố/mở lại ghi audit log (người, lúc, lý do). BR-S4-10: chỉ học viên còn BOOKED lúc lớp kết thúc có tổng kết; học viên đã huỷ/đổi lớp không có (học viên đổi sang lớp khác được tổng kết ở lớp mới).</t>
+  </si>
+  <si>
+    <t>POST /classes/:id/summary/publish, POST /classes/:id/summary/reopen</t>
+  </si>
+  <si>
+    <t>S4-15</t>
+  </si>
+  <si>
+    <t>FE – Công bố / mở lại tổng kết: HLV bấm Công bố → khoá bản tổng kết, gửi thông báo in-app + email cho từng học viên. Sau khi công bố chỉ quản lý được mở lại (nhập lý do), HLV sửa và công bố lại thì hội viên nhận thông báo cập nhật.</t>
+  </si>
+  <si>
+    <t>11/11/2026</t>
+  </si>
+  <si>
+    <t>Nút Công bố + hộp xác nhận cảnh báo buổi chưa điểm danh; nút Mở lại cho quản lý · Khải hoàn thiện 29/10/2026 trên sprint-4/fe-khai; bàn giao docs/handover/sprint-4-fe-khai.md. Đã xác minh 238 BE, 160 FE và đủ 86 E2E desktop sau chạy lại; 15 test case bổ sung, chờ leader review.</t>
+  </si>
+  <si>
+    <t>S4-16</t>
+  </si>
+  <si>
+    <t>UC-TR-06</t>
+  </si>
+  <si>
+    <t>BE – Hội viên xem kết quả khoá học (màn S38 mới, trong Hồ sơ → "Khoá học đã hoàn thành"): danh sách khoá đã kết thúc, chuyên cần, kết quả, mức tiến bộ, nhận xét của HLV, gợi ý khoá tiếp; tải "Phiếu tổng kết khoá học" PDF.</t>
+  </si>
+  <si>
+    <t>Chỉ thấy tổng kết đã công bố của chính mình. PDF dùng lại khung mẫu hoá đơn PDF (UC-PAY-07): logo, thông tin trung tâm, khoá, HLV, chuyên cần, kết quả, nhận xét, mã tra cứu.</t>
+  </si>
+  <si>
+    <t>GET /me/course-results, GET /me/course-results/:id/pdf</t>
+  </si>
+  <si>
+    <t>S4-17</t>
+  </si>
+  <si>
+    <t>FE – Hội viên xem kết quả khoá học (màn S38 mới, trong Hồ sơ → "Khoá học đã hoàn thành"): danh sách khoá đã kết thúc, chuyên cần, kết quả, mức tiến bộ, nhận xét của HLV, gợi ý khoá tiếp; tải "Phiếu tổng kết khoá học" PDF.</t>
+  </si>
+  <si>
+    <t>Mục "Khoá học đã hoàn thành" trong Hồ sơ (S38) · Khải hoàn thiện 29/10/2026 trên sprint-4/fe-khai; bàn giao docs/handover/sprint-4-fe-khai.md. Đã xác minh 238 BE, 160 FE và đủ 86 E2E desktop sau chạy lại; 15 test case bổ sung, chờ leader review.</t>
+  </si>
+  <si>
+    <t>S4-18</t>
+  </si>
+  <si>
+    <t>UC-TR-07</t>
+  </si>
+  <si>
+    <t>BE – Hội viên đánh giá khoá học và HLV: sau khi khoá kết thúc, hội viên chấm 1–5 sao cho khoá và cho HLV kèm nhận xét; sửa được trong thời hạn. Điểm trung bình hiện ở hồ sơ HLV (UC-UM-23) và báo cáo tổng kết khoá (UC-RPT-03).</t>
+  </si>
+  <si>
+    <t>BR-S4-11: chỉ học viên có tổng kết ở lớp đó; mỗi học viên một đánh giá mỗi lớp; trong COURSE_RATING_WINDOW_DAYS (14) ngày kể từ khi lớp kết thúc. HLV thấy điểm và nhận xét ẩn danh; quản lý thấy tên người đánh giá và ẩn được nhận xét không phù hợp (audit log).</t>
+  </si>
+  <si>
+    <t>POST/PUT /classes/:id/ratings, GET /coaches/:id/ratings</t>
+  </si>
+  <si>
+    <t>S4-19</t>
+  </si>
+  <si>
+    <t>FE – Hội viên đánh giá khoá học và HLV: sau khi khoá kết thúc, hội viên chấm 1–5 sao cho khoá và cho HLV kèm nhận xét; sửa được trong thời hạn. Điểm trung bình hiện ở hồ sơ HLV (UC-UM-23) và báo cáo tổng kết khoá (UC-RPT-03).</t>
+  </si>
+  <si>
+    <t>13/11/2026</t>
+  </si>
+  <si>
+    <t>Form đánh giá trong S38; khối đánh giá trên hồ sơ HLV phối hợp với Khôi · Khải hoàn thiện 29/10/2026 trên sprint-4/fe-khai; bàn giao docs/handover/sprint-4-fe-khai.md. Đã xác minh 238 BE, 160 FE và đủ 86 E2E desktop sau chạy lại; 15 test case bổ sung, chờ leader review.</t>
+  </si>
+  <si>
+    <t>S4-20</t>
+  </si>
+  <si>
+    <t>UC-RPT-03</t>
+  </si>
+  <si>
+    <t>BE – Báo cáo tổng kết khoá cho quản lý (màn S39 mới, tab trong Báo cáo): danh sách khoá kết thúc trong khoảng thời gian; tỉ lệ hoàn thành, chuyên cần trung bình, % Đạt, điểm đánh giá trung bình; lọc theo bộ môn, HLV; đánh dấu khoá HLV chưa nộp tổng kết; xuất Excel.</t>
+  </si>
+  <si>
+    <t>Quyền COURSE_SUMMARY_VIEW_ALL (report.view không đủ). Khoảng thời gian tối đa theo REPORT_MAX_DAYS hiện có. Số liệu từ cùng một truy vấn cho màn hình và file xuất.</t>
+  </si>
+  <si>
+    <t>GET /reports/course-summaries + xuất Excel</t>
+  </si>
+  <si>
+    <t>S4-21</t>
+  </si>
+  <si>
+    <t>FE – Báo cáo tổng kết khoá cho quản lý (màn S39 mới, tab trong Báo cáo): danh sách khoá kết thúc trong khoảng thời gian; tỉ lệ hoàn thành, chuyên cần trung bình, % Đạt, điểm đánh giá trung bình; lọc theo bộ môn, HLV; đánh dấu khoá HLV chưa nộp tổng kết; xuất Excel.</t>
+  </si>
+  <si>
+    <t>14/11/2026</t>
+  </si>
+  <si>
+    <t>Tab "Tổng kết khoá" trong trang Báo cáo · Khải hoàn thiện 29/10/2026 trên sprint-4/fe-khai; bàn giao docs/handover/sprint-4-fe-khai.md. Đã xác minh 238 BE, 160 FE và đủ 86 E2E desktop sau chạy lại; 15 test case bổ sung, chờ leader review.</t>
+  </si>
+  <si>
+    <t>S4-22</t>
+  </si>
+  <si>
+    <t>UC-RPT-02</t>
+  </si>
+  <si>
+    <t>BE – Doanh thu theo thời gian (màn 17 mở rộng): chọn nhóm theo ngày / tuần / tháng / quý / năm và khoảng nhanh (hôm nay, 7 ngày, tháng này, quý này, năm nay, tuỳ chọn); biểu đồ cột thu – hoàn – thuần theo từng kỳ, bảng số liệu bên dưới.</t>
+  </si>
+  <si>
+    <t>BR-S4-12: ghi nhận doanh thu theo ngày thanh toán (paidAt), hoàn theo ngày hoàn (completedAt), múi giờ Việt Nam, tuần bắt đầu thứ Hai. Phần trả bằng số dư không tính lại (BR-GY-13). BR-S4-14: giới hạn khoảng theo nhóm đọc từ cấu hình: ngày ≤ 92 ngày, tuần ≤ 1 năm, tháng/quý/năm ≤ 5 năm.</t>
+  </si>
+  <si>
+    <t>Tham số groupBy=day|week|month|quarter|year; hàm chia kỳ dùng chung cho #123 · Chuyển từ Nhanh sang Bảo theo phân công 29/10/2026.</t>
+  </si>
+  <si>
+    <t>S4-23</t>
+  </si>
+  <si>
+    <t>FE – Doanh thu theo thời gian (màn 17 mở rộng): chọn nhóm theo ngày / tuần / tháng / quý / năm và khoảng nhanh (hôm nay, 7 ngày, tháng này, quý này, năm nay, tuỳ chọn); biểu đồ cột thu – hoàn – thuần theo từng kỳ, bảng số liệu bên dưới.</t>
+  </si>
+  <si>
+    <t>Bộ chọn nhóm + khoảng nhanh, biểu đồ cột · Chuyển từ Nhanh sang Bảo theo phân công 29/10/2026.</t>
+  </si>
+  <si>
+    <t>S4-24</t>
+  </si>
+  <si>
+    <t>BE – So sánh kỳ trước và cơ cấu doanh thu: % tăng/giảm so với khoảng liền trước cùng độ dài; tách doanh thu theo loại (gói tự tập / khoá học / chênh lệch đổi), theo kênh (online / tại quầy); top gói tự tập, top lớp và theo bộ môn.</t>
+  </si>
+  <si>
+    <t>BR-S4-13: kỳ trước bằng 0 thì hiện "—" thay vì vô cực. BR-S4-15: tổng các phần cơ cấu phải bằng doanh thu thuần của kỳ (có test BE). Hoá đơn ADJUSTMENT tính vào nhóm "chênh lệch", không cộng vào gói/khoá gốc.</t>
+  </si>
+  <si>
+    <t>compare=previous, breakdown theo loại hoá đơn/kênh/gói/lớp/bộ môn · Chuyển từ Nhanh sang Bảo theo phân công 29/10/2026.</t>
+  </si>
+  <si>
+    <t>S4-25</t>
+  </si>
+  <si>
+    <t>FE – So sánh kỳ trước và cơ cấu doanh thu: % tăng/giảm so với khoảng liền trước cùng độ dài; tách doanh thu theo loại (gói tự tập / khoá học / chênh lệch đổi), theo kênh (online / tại quầy); top gói tự tập, top lớp và theo bộ môn.</t>
+  </si>
+  <si>
+    <t>Thẻ KPI có % so với kỳ trước, biểu đồ cơ cấu, bảng top · Chuyển từ Nhanh sang Bảo theo phân công 29/10/2026.</t>
+  </si>
+  <si>
+    <t>S4-26</t>
+  </si>
+  <si>
+    <t>UC-RPT-04</t>
+  </si>
+  <si>
+    <t>BE – Báo cáo hội viên và đăng ký theo thời gian (màn 17, tab mới): theo cùng nhóm ngày/tuần/tháng/quý/năm — số hội viên mới, kỳ gói đang hiệu lực, đăng ký khoá học mới, số huỷ gói/huỷ khoá, tỉ lệ lấp đầy lớp.</t>
+  </si>
+  <si>
+    <t>Đáp ứng yêu cầu đề tài "báo cáo số lượng thành viên, tình trạng đăng ký lớp và doanh thu theo thời gian". Dùng chung bộ lọc và hàm chia kỳ với UC-RPT-02 (không viết lại).</t>
+  </si>
+  <si>
+    <t>Tách file report-member.service.js, dùng hàm chia kỳ của S4-22</t>
+  </si>
+  <si>
+    <t>S4-27</t>
+  </si>
+  <si>
+    <t>FE – Báo cáo hội viên và đăng ký theo thời gian (màn 17, tab mới): theo cùng nhóm ngày/tuần/tháng/quý/năm — số hội viên mới, kỳ gói đang hiệu lực, đăng ký khoá học mới, số huỷ gói/huỷ khoá, tỉ lệ lấp đầy lớp.</t>
+  </si>
+  <si>
+    <t>Tab "Hội viên &amp; đăng ký" trong Báo cáo · Chuyển từ Nhanh sang Bảo theo phân công 29/10/2026.</t>
+  </si>
+  <si>
+    <t>S4-28</t>
+  </si>
+  <si>
+    <t>UC-RPT-01</t>
+  </si>
+  <si>
+    <t>BE – Xuất báo cáo theo nhóm thời gian (sửa UC-RPT-01): PDF/CSV/Excel giữ đúng nhóm kỳ, phần so sánh kỳ trước và cơ cấu doanh thu như trên màn hình.</t>
+  </si>
+  <si>
+    <t>Cùng dữ liệu và công thức với dashboard (một hàm build dùng chung, như buildRevenue hiện tại).</t>
+  </si>
+  <si>
+    <t>Sửa report-export.service.js · Chuyển từ Nhanh sang Bảo theo phân công 29/10/2026.</t>
+  </si>
+  <si>
+    <t>S4-29</t>
+  </si>
+  <si>
+    <t>Kiểm thử</t>
+  </si>
+  <si>
+    <t>Kiểm thử – E2E Playwright tổng kết khoá, đánh giá, báo cáo doanh thu theo thời gian, xuất file.</t>
+  </si>
+  <si>
+    <t>Test</t>
+  </si>
+  <si>
+    <t>Chạy trên npm run db:demo; E2E cũ phải pass.</t>
+  </si>
+  <si>
+    <t>15/11/2026</t>
+  </si>
+  <si>
+    <t>#125 · Khải hoàn thiện 29/10/2026 trên sprint-4/fe-khai; bàn giao docs/handover/sprint-4-fe-khai.md. Đã xác minh 238 BE, 160 FE và đủ 86 E2E desktop sau chạy lại; 15 test case bổ sung, chờ leader review.</t>
+  </si>
+  <si>
+    <t>S4-30</t>
+  </si>
+  <si>
+    <t>Kiểm thử – E2E Playwright hồ sơ HLV, hồ sơ hội viên, HLV xem hồ sơ học viên (trong và ngoài phạm vi).</t>
+  </si>
+  <si>
+    <t>BR-S4-03: kiểm tra 403 khi HLV mở hồ sơ hội viên không học lớp mình.</t>
+  </si>
+  <si>
+    <t>#125 · Khôi hoàn thiện hồ sơ BE/FE và kiểm thử ngày 29/10/2026; bàn giao tại docs/handover/sprint-4-fe-khoi.md.</t>
+  </si>
+  <si>
+    <t>S4-31</t>
+  </si>
+  <si>
+    <t>Kiểm thử – Bổ sung test case Sprint 4 vào docs/kiem-thu/SWP391_TestCase.xlsx và ghi kết quả chạy.</t>
+  </si>
+  <si>
+    <t>—</t>
+  </si>
+  <si>
+    <t>Khôi viết phần hồ sơ, Khải phần còn lại. #125 · Khải hoàn thiện 29/10/2026 trên sprint-4/fe-khai; bàn giao docs/handover/sprint-4-fe-khai.md. Đã xác minh 238 BE, 160 FE và đủ 86 E2E desktop sau chạy lại; 15 test case bổ sung, chờ leader review.</t>
+  </si>
+  <si>
+    <t>S4-32</t>
+  </si>
+  <si>
+    <t>Tài liệu</t>
+  </si>
+  <si>
+    <t>Tài liệu – Đặc tả UC-UM-22…25, UC-TR-05…07, UC-RPT-02…04, BR-S4-01…15 vào docs/yeu-cau; ERD bổ sung.</t>
+  </si>
+  <si>
+    <t>Docs</t>
+  </si>
+  <si>
+    <t>#126</t>
+  </si>
+  <si>
+    <t>S4-33</t>
+  </si>
+  <si>
+    <t>Tài liệu – Seed demo Sprint 4: khoá đã kết thúc có/chưa có tổng kết, đánh giá, hồ sơ HLV/hội viên đầy đủ, doanh thu rải 12 tháng để xem theo tháng/quý.</t>
+  </si>
+  <si>
+    <t>#126 · Chuyển từ Nhanh sang Bảo theo phân công 29/10/2026.</t>
+  </si>
+  <si>
+    <t>S4-34</t>
+  </si>
+  <si>
+    <t>Tài liệu – Kịch bản demo cuối kỳ (cập nhật LoTrinh_Demo) và diễn tập cả nhóm.</t>
+  </si>
+  <si>
+    <t>In Progress</t>
+  </si>
+  <si>
+    <t>#126. Khoá code 16/11. · Chuyển từ Nhanh sang Bảo theo phân công 29/10/2026. · Đã chuẩn bị kịch bản và test tự động; chờ diễn tập trực tiếp cả nhóm sau tích hợp Khôi/Khải.</t>
+  </si>
+  <si>
+    <t>Tiến độ Sprint 4 theo thành viên</t>
+  </si>
+  <si>
+    <t>Thành viên</t>
+  </si>
+  <si>
+    <t>Vai</t>
+  </si>
+  <si>
+    <t>Tổng task</t>
+  </si>
+  <si>
     <t>To Do</t>
-  </si>
-  <si>
-    <t>Màn S37, làm theo contract trước, giả lập dữ liệu nếu BE chưa xong</t>
-  </si>
-  <si>
-    <t>S4-14</t>
-  </si>
-  <si>
-    <t>BE – Công bố / mở lại tổng kết: HLV bấm Công bố → khoá bản tổng kết, gửi thông báo in-app + email cho từng học viên. Sau khi công bố chỉ quản lý được mở lại (nhập lý do), HLV sửa và công bố lại thì hội viên nhận thông báo cập nhật.</t>
-  </si>
-  <si>
-    <t>BR-S4-09: chỉ công bố khi mọi học viên đã có kết quả. Công bố/mở lại ghi audit log (người, lúc, lý do). BR-S4-10: chỉ học viên còn BOOKED lúc lớp kết thúc có tổng kết; học viên đã huỷ/đổi lớp không có (học viên đổi sang lớp khác được tổng kết ở lớp mới).</t>
-  </si>
-  <si>
-    <t>POST /classes/:id/summary/publish, POST /classes/:id/summary/reopen</t>
-  </si>
-  <si>
-    <t>S4-15</t>
-  </si>
-  <si>
-    <t>FE – Công bố / mở lại tổng kết: HLV bấm Công bố → khoá bản tổng kết, gửi thông báo in-app + email cho từng học viên. Sau khi công bố chỉ quản lý được mở lại (nhập lý do), HLV sửa và công bố lại thì hội viên nhận thông báo cập nhật.</t>
-  </si>
-  <si>
-    <t>11/11/2026</t>
-  </si>
-  <si>
-    <t>Nút Công bố + hộp xác nhận cảnh báo buổi chưa điểm danh; nút Mở lại cho quản lý</t>
-  </si>
-  <si>
-    <t>S4-16</t>
-  </si>
-  <si>
-    <t>UC-TR-06</t>
-  </si>
-  <si>
-    <t>BE – Hội viên xem kết quả khoá học (màn S38 mới, trong Hồ sơ → "Khoá học đã hoàn thành"): danh sách khoá đã kết thúc, chuyên cần, kết quả, mức tiến bộ, nhận xét của HLV, gợi ý khoá tiếp; tải "Phiếu tổng kết khoá học" PDF.</t>
-  </si>
-  <si>
-    <t>Chỉ thấy tổng kết đã công bố của chính mình. PDF dùng lại khung mẫu hoá đơn PDF (UC-PAY-07): logo, thông tin trung tâm, khoá, HLV, chuyên cần, kết quả, nhận xét, mã tra cứu.</t>
-  </si>
-  <si>
-    <t>GET /me/course-results, GET /me/course-results/:id/pdf</t>
-  </si>
-  <si>
-    <t>S4-17</t>
-  </si>
-  <si>
-    <t>FE – Hội viên xem kết quả khoá học (màn S38 mới, trong Hồ sơ → "Khoá học đã hoàn thành"): danh sách khoá đã kết thúc, chuyên cần, kết quả, mức tiến bộ, nhận xét của HLV, gợi ý khoá tiếp; tải "Phiếu tổng kết khoá học" PDF.</t>
-  </si>
-  <si>
-    <t>Mục "Khoá học đã hoàn thành" trong Hồ sơ (S38)</t>
-  </si>
-  <si>
-    <t>S4-18</t>
-  </si>
-  <si>
-    <t>UC-TR-07</t>
-  </si>
-  <si>
-    <t>BE – Hội viên đánh giá khoá học và HLV: sau khi khoá kết thúc, hội viên chấm 1–5 sao cho khoá và cho HLV kèm nhận xét; sửa được trong thời hạn. Điểm trung bình hiện ở hồ sơ HLV (UC-UM-23) và báo cáo tổng kết khoá (UC-RPT-03).</t>
-  </si>
-  <si>
-    <t>BR-S4-11: chỉ học viên có tổng kết ở lớp đó; mỗi học viên một đánh giá mỗi lớp; trong COURSE_RATING_WINDOW_DAYS (14) ngày kể từ khi lớp kết thúc. HLV thấy điểm và nhận xét ẩn danh; quản lý thấy tên người đánh giá và ẩn được nhận xét không phù hợp (audit log).</t>
-  </si>
-  <si>
-    <t>POST/PUT /classes/:id/ratings, GET /coaches/:id/ratings</t>
-  </si>
-  <si>
-    <t>S4-19</t>
-  </si>
-  <si>
-    <t>FE – Hội viên đánh giá khoá học và HLV: sau khi khoá kết thúc, hội viên chấm 1–5 sao cho khoá và cho HLV kèm nhận xét; sửa được trong thời hạn. Điểm trung bình hiện ở hồ sơ HLV (UC-UM-23) và báo cáo tổng kết khoá (UC-RPT-03).</t>
-  </si>
-  <si>
-    <t>13/11/2026</t>
-  </si>
-  <si>
-    <t>Form đánh giá trong S38; khối đánh giá trên hồ sơ HLV phối hợp với Khôi</t>
-  </si>
-  <si>
-    <t>S4-20</t>
-  </si>
-  <si>
-    <t>UC-RPT-03</t>
-  </si>
-  <si>
-    <t>BE – Báo cáo tổng kết khoá cho quản lý (màn S39 mới, tab trong Báo cáo): danh sách khoá kết thúc trong khoảng thời gian; tỉ lệ hoàn thành, chuyên cần trung bình, % Đạt, điểm đánh giá trung bình; lọc theo bộ môn, HLV; đánh dấu khoá HLV chưa nộp tổng kết; xuất Excel.</t>
-  </si>
-  <si>
-    <t>Quyền COURSE_SUMMARY_VIEW_ALL (report.view không đủ). Khoảng thời gian tối đa theo REPORT_MAX_DAYS hiện có. Số liệu từ cùng một truy vấn cho màn hình và file xuất.</t>
-  </si>
-  <si>
-    <t>GET /reports/course-summaries + xuất Excel</t>
-  </si>
-  <si>
-    <t>S4-21</t>
-  </si>
-  <si>
-    <t>FE – Báo cáo tổng kết khoá cho quản lý (màn S39 mới, tab trong Báo cáo): danh sách khoá kết thúc trong khoảng thời gian; tỉ lệ hoàn thành, chuyên cần trung bình, % Đạt, điểm đánh giá trung bình; lọc theo bộ môn, HLV; đánh dấu khoá HLV chưa nộp tổng kết; xuất Excel.</t>
-  </si>
-  <si>
-    <t>14/11/2026</t>
-  </si>
-  <si>
-    <t>Tab "Tổng kết khoá" trong trang Báo cáo</t>
-  </si>
-  <si>
-    <t>S4-22</t>
-  </si>
-  <si>
-    <t>UC-RPT-02</t>
-  </si>
-  <si>
-    <t>BE – Doanh thu theo thời gian (màn 17 mở rộng): chọn nhóm theo ngày / tuần / tháng / quý / năm và khoảng nhanh (hôm nay, 7 ngày, tháng này, quý này, năm nay, tuỳ chọn); biểu đồ cột thu – hoàn – thuần theo từng kỳ, bảng số liệu bên dưới.</t>
-  </si>
-  <si>
-    <t>BR-S4-12: ghi nhận doanh thu theo ngày thanh toán (paidAt), hoàn theo ngày hoàn (completedAt), múi giờ Việt Nam, tuần bắt đầu thứ Hai. Phần trả bằng số dư không tính lại (BR-GY-13). BR-S4-14: giới hạn khoảng theo nhóm đọc từ cấu hình: ngày ≤ 92 ngày, tuần ≤ 1 năm, tháng/quý/năm ≤ 5 năm.</t>
-  </si>
-  <si>
-    <t>Tham số groupBy=day|week|month|quarter|year; hàm chia kỳ dùng chung cho #123 · Chuyển từ Nhanh sang Bảo theo phân công 29/10/2026.</t>
-  </si>
-  <si>
-    <t>S4-23</t>
-  </si>
-  <si>
-    <t>FE – Doanh thu theo thời gian (màn 17 mở rộng): chọn nhóm theo ngày / tuần / tháng / quý / năm và khoảng nhanh (hôm nay, 7 ngày, tháng này, quý này, năm nay, tuỳ chọn); biểu đồ cột thu – hoàn – thuần theo từng kỳ, bảng số liệu bên dưới.</t>
-  </si>
-  <si>
-    <t>Bộ chọn nhóm + khoảng nhanh, biểu đồ cột · Chuyển từ Nhanh sang Bảo theo phân công 29/10/2026.</t>
-  </si>
-  <si>
-    <t>S4-24</t>
-  </si>
-  <si>
-    <t>BE – So sánh kỳ trước và cơ cấu doanh thu: % tăng/giảm so với khoảng liền trước cùng độ dài; tách doanh thu theo loại (gói tự tập / khoá học / chênh lệch đổi), theo kênh (online / tại quầy); top gói tự tập, top lớp và theo bộ môn.</t>
-  </si>
-  <si>
-    <t>BR-S4-13: kỳ trước bằng 0 thì hiện "—" thay vì vô cực. BR-S4-15: tổng các phần cơ cấu phải bằng doanh thu thuần của kỳ (có test BE). Hoá đơn ADJUSTMENT tính vào nhóm "chênh lệch", không cộng vào gói/khoá gốc.</t>
-  </si>
-  <si>
-    <t>compare=previous, breakdown theo loại hoá đơn/kênh/gói/lớp/bộ môn · Chuyển từ Nhanh sang Bảo theo phân công 29/10/2026.</t>
-  </si>
-  <si>
-    <t>S4-25</t>
-  </si>
-  <si>
-    <t>FE – So sánh kỳ trước và cơ cấu doanh thu: % tăng/giảm so với khoảng liền trước cùng độ dài; tách doanh thu theo loại (gói tự tập / khoá học / chênh lệch đổi), theo kênh (online / tại quầy); top gói tự tập, top lớp và theo bộ môn.</t>
-  </si>
-  <si>
-    <t>Thẻ KPI có % so với kỳ trước, biểu đồ cơ cấu, bảng top · Chuyển từ Nhanh sang Bảo theo phân công 29/10/2026.</t>
-  </si>
-  <si>
-    <t>S4-26</t>
-  </si>
-  <si>
-    <t>UC-RPT-04</t>
-  </si>
-  <si>
-    <t>BE – Báo cáo hội viên và đăng ký theo thời gian (màn 17, tab mới): theo cùng nhóm ngày/tuần/tháng/quý/năm — số hội viên mới, kỳ gói đang hiệu lực, đăng ký khoá học mới, số huỷ gói/huỷ khoá, tỉ lệ lấp đầy lớp.</t>
-  </si>
-  <si>
-    <t>Đáp ứng yêu cầu đề tài "báo cáo số lượng thành viên, tình trạng đăng ký lớp và doanh thu theo thời gian". Dùng chung bộ lọc và hàm chia kỳ với UC-RPT-02 (không viết lại).</t>
-  </si>
-  <si>
-    <t>Tách file report-member.service.js, dùng hàm chia kỳ của S4-22</t>
-  </si>
-  <si>
-    <t>S4-27</t>
-  </si>
-  <si>
-    <t>FE – Báo cáo hội viên và đăng ký theo thời gian (màn 17, tab mới): theo cùng nhóm ngày/tuần/tháng/quý/năm — số hội viên mới, kỳ gói đang hiệu lực, đăng ký khoá học mới, số huỷ gói/huỷ khoá, tỉ lệ lấp đầy lớp.</t>
-  </si>
-  <si>
-    <t>Tab "Hội viên &amp; đăng ký" trong Báo cáo · Chuyển từ Nhanh sang Bảo theo phân công 29/10/2026.</t>
-  </si>
-  <si>
-    <t>S4-28</t>
-  </si>
-  <si>
-    <t>UC-RPT-01</t>
-  </si>
-  <si>
-    <t>BE – Xuất báo cáo theo nhóm thời gian (sửa UC-RPT-01): PDF/CSV/Excel giữ đúng nhóm kỳ, phần so sánh kỳ trước và cơ cấu doanh thu như trên màn hình.</t>
-  </si>
-  <si>
-    <t>Cùng dữ liệu và công thức với dashboard (một hàm build dùng chung, như buildRevenue hiện tại).</t>
-  </si>
-  <si>
-    <t>Sửa report-export.service.js · Chuyển từ Nhanh sang Bảo theo phân công 29/10/2026.</t>
-  </si>
-  <si>
-    <t>S4-29</t>
-  </si>
-  <si>
-    <t>Kiểm thử</t>
-  </si>
-  <si>
-    <t>Kiểm thử – E2E Playwright tổng kết khoá, đánh giá, báo cáo doanh thu theo thời gian, xuất file.</t>
-  </si>
-  <si>
-    <t>Test</t>
-  </si>
-  <si>
-    <t>Chạy trên npm run db:demo; E2E cũ phải pass.</t>
-  </si>
-  <si>
-    <t>15/11/2026</t>
-  </si>
-  <si>
-    <t>#125</t>
-  </si>
-  <si>
-    <t>S4-30</t>
-  </si>
-  <si>
-    <t>Kiểm thử – E2E Playwright hồ sơ HLV, hồ sơ hội viên, HLV xem hồ sơ học viên (trong và ngoài phạm vi).</t>
-  </si>
-  <si>
-    <t>BR-S4-03: kiểm tra 403 khi HLV mở hồ sơ hội viên không học lớp mình.</t>
-  </si>
-  <si>
-    <t>#125 · Khôi hoàn thiện hồ sơ BE/FE và kiểm thử ngày 29/10/2026; bàn giao tại docs/handover/sprint-4-fe-khoi.md.</t>
-  </si>
-  <si>
-    <t>S4-31</t>
-  </si>
-  <si>
-    <t>Kiểm thử – Bổ sung test case Sprint 4 vào docs/kiem-thu/SWP391_TestCase.xlsx và ghi kết quả chạy.</t>
-  </si>
-  <si>
-    <t>—</t>
-  </si>
-  <si>
-    <t>Khôi viết phần hồ sơ, Khải phần còn lại. #125</t>
-  </si>
-  <si>
-    <t>S4-32</t>
-  </si>
-  <si>
-    <t>Tài liệu</t>
-  </si>
-  <si>
-    <t>Tài liệu – Đặc tả UC-UM-22…25, UC-TR-05…07, UC-RPT-02…04, BR-S4-01…15 vào docs/yeu-cau; ERD bổ sung.</t>
-  </si>
-  <si>
-    <t>Docs</t>
-  </si>
-  <si>
-    <t>#126</t>
-  </si>
-  <si>
-    <t>S4-33</t>
-  </si>
-  <si>
-    <t>Tài liệu – Seed demo Sprint 4: khoá đã kết thúc có/chưa có tổng kết, đánh giá, hồ sơ HLV/hội viên đầy đủ, doanh thu rải 12 tháng để xem theo tháng/quý.</t>
-  </si>
-  <si>
-    <t>#126 · Chuyển từ Nhanh sang Bảo theo phân công 29/10/2026.</t>
-  </si>
-  <si>
-    <t>S4-34</t>
-  </si>
-  <si>
-    <t>Tài liệu – Kịch bản demo cuối kỳ (cập nhật LoTrinh_Demo) và diễn tập cả nhóm.</t>
-  </si>
-  <si>
-    <t>In Progress</t>
-  </si>
-  <si>
-    <t>#126. Khoá code 16/11. · Chuyển từ Nhanh sang Bảo theo phân công 29/10/2026. · Đã chuẩn bị kịch bản và test tự động; chờ diễn tập trực tiếp cả nhóm sau tích hợp Khôi/Khải.</t>
-  </si>
-  <si>
-    <t>Tiến độ Sprint 4 theo thành viên</t>
-  </si>
-  <si>
-    <t>Thành viên</t>
-  </si>
-  <si>
-    <t>Vai</t>
-  </si>
-  <si>
-    <t>Tổng task</t>
   </si>
   <si>
     <t>Done</t>
@@ -1691,21 +1691,21 @@
         <v>57</v>
       </c>
       <c r="K18" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="L18" s="7" t="s">
         <v>90</v>
-      </c>
-      <c r="L18" s="7" t="s">
-        <v>91</v>
       </c>
     </row>
     <row r="19" ht="60" customHeight="1" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A19" s="6" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B19" s="6" t="s">
         <v>77</v>
       </c>
       <c r="C19" s="7" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D19" s="8" t="s">
         <v>17</v>
@@ -1717,7 +1717,7 @@
         <v>19</v>
       </c>
       <c r="G19" s="7" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="H19" s="6" t="s">
         <v>21</v>
@@ -1732,18 +1732,18 @@
         <v>24</v>
       </c>
       <c r="L19" s="7" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="20" ht="60" customHeight="1" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A20" s="6" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B20" s="6" t="s">
         <v>77</v>
       </c>
       <c r="C20" s="7" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="D20" s="8" t="s">
         <v>36</v>
@@ -1755,7 +1755,7 @@
         <v>19</v>
       </c>
       <c r="G20" s="7" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="H20" s="6" t="s">
         <v>89</v>
@@ -1764,24 +1764,24 @@
         <v>53</v>
       </c>
       <c r="J20" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="K20" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="L20" s="7" t="s">
         <v>98</v>
-      </c>
-      <c r="K20" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="L20" s="7" t="s">
-        <v>99</v>
       </c>
     </row>
     <row r="21" ht="60" customHeight="1" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A21" s="6" t="s">
+        <v>99</v>
+      </c>
+      <c r="B21" s="6" t="s">
         <v>100</v>
       </c>
-      <c r="B21" s="6" t="s">
+      <c r="C21" s="7" t="s">
         <v>101</v>
-      </c>
-      <c r="C21" s="7" t="s">
-        <v>102</v>
       </c>
       <c r="D21" s="8" t="s">
         <v>17</v>
@@ -1793,7 +1793,7 @@
         <v>19</v>
       </c>
       <c r="G21" s="7" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="H21" s="6" t="s">
         <v>21</v>
@@ -1802,24 +1802,24 @@
         <v>53</v>
       </c>
       <c r="J21" s="6" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="K21" s="6" t="s">
         <v>24</v>
       </c>
       <c r="L21" s="7" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="22" ht="60" customHeight="1" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A22" s="6" t="s">
+        <v>104</v>
+      </c>
+      <c r="B22" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="C22" s="7" t="s">
         <v>105</v>
-      </c>
-      <c r="B22" s="6" t="s">
-        <v>101</v>
-      </c>
-      <c r="C22" s="7" t="s">
-        <v>106</v>
       </c>
       <c r="D22" s="8" t="s">
         <v>36</v>
@@ -1831,7 +1831,7 @@
         <v>19</v>
       </c>
       <c r="G22" s="7" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="H22" s="6" t="s">
         <v>89</v>
@@ -1843,21 +1843,21 @@
         <v>74</v>
       </c>
       <c r="K22" s="6" t="s">
-        <v>90</v>
+        <v>24</v>
       </c>
       <c r="L22" s="7" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="23" ht="60" customHeight="1" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A23" s="6" t="s">
+        <v>107</v>
+      </c>
+      <c r="B23" s="6" t="s">
         <v>108</v>
       </c>
-      <c r="B23" s="6" t="s">
+      <c r="C23" s="7" t="s">
         <v>109</v>
-      </c>
-      <c r="C23" s="7" t="s">
-        <v>110</v>
       </c>
       <c r="D23" s="8" t="s">
         <v>17</v>
@@ -1869,7 +1869,7 @@
         <v>19</v>
       </c>
       <c r="G23" s="7" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="H23" s="6" t="s">
         <v>21</v>
@@ -1884,18 +1884,18 @@
         <v>24</v>
       </c>
       <c r="L23" s="7" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="24" ht="60" customHeight="1" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A24" s="6" t="s">
+        <v>112</v>
+      </c>
+      <c r="B24" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="C24" s="7" t="s">
         <v>113</v>
-      </c>
-      <c r="B24" s="6" t="s">
-        <v>109</v>
-      </c>
-      <c r="C24" s="7" t="s">
-        <v>114</v>
       </c>
       <c r="D24" s="8" t="s">
         <v>36</v>
@@ -1907,33 +1907,33 @@
         <v>19</v>
       </c>
       <c r="G24" s="7" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="H24" s="6" t="s">
         <v>89</v>
       </c>
       <c r="I24" s="6" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="J24" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="K24" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="L24" s="7" t="s">
         <v>115</v>
-      </c>
-      <c r="K24" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="L24" s="7" t="s">
-        <v>116</v>
       </c>
     </row>
     <row r="25" ht="60" customHeight="1" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A25" s="6" t="s">
+        <v>116</v>
+      </c>
+      <c r="B25" s="6" t="s">
         <v>117</v>
       </c>
-      <c r="B25" s="6" t="s">
+      <c r="C25" s="7" t="s">
         <v>118</v>
-      </c>
-      <c r="C25" s="7" t="s">
-        <v>119</v>
       </c>
       <c r="D25" s="8" t="s">
         <v>17</v>
@@ -1945,33 +1945,33 @@
         <v>19</v>
       </c>
       <c r="G25" s="7" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="H25" s="6" t="s">
         <v>21</v>
       </c>
       <c r="I25" s="6" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="J25" s="6" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="K25" s="6" t="s">
         <v>24</v>
       </c>
       <c r="L25" s="7" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="26" ht="60" customHeight="1" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A26" s="6" t="s">
+        <v>121</v>
+      </c>
+      <c r="B26" s="6" t="s">
+        <v>117</v>
+      </c>
+      <c r="C26" s="7" t="s">
         <v>122</v>
-      </c>
-      <c r="B26" s="6" t="s">
-        <v>118</v>
-      </c>
-      <c r="C26" s="7" t="s">
-        <v>123</v>
       </c>
       <c r="D26" s="8" t="s">
         <v>36</v>
@@ -1983,7 +1983,7 @@
         <v>19</v>
       </c>
       <c r="G26" s="7" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="H26" s="6" t="s">
         <v>89</v>
@@ -1992,24 +1992,24 @@
         <v>74</v>
       </c>
       <c r="J26" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="K26" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="L26" s="7" t="s">
         <v>124</v>
-      </c>
-      <c r="K26" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="L26" s="7" t="s">
-        <v>125</v>
       </c>
     </row>
     <row r="27" ht="60" customHeight="1" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A27" s="6" t="s">
+        <v>125</v>
+      </c>
+      <c r="B27" s="6" t="s">
         <v>126</v>
       </c>
-      <c r="B27" s="6" t="s">
+      <c r="C27" s="7" t="s">
         <v>127</v>
-      </c>
-      <c r="C27" s="7" t="s">
-        <v>128</v>
       </c>
       <c r="D27" s="8" t="s">
         <v>17</v>
@@ -2021,7 +2021,7 @@
         <v>19</v>
       </c>
       <c r="G27" s="7" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="H27" s="6" t="s">
         <v>21</v>
@@ -2036,18 +2036,18 @@
         <v>24</v>
       </c>
       <c r="L27" s="7" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="28" ht="60" customHeight="1" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A28" s="6" t="s">
+        <v>130</v>
+      </c>
+      <c r="B28" s="6" t="s">
+        <v>126</v>
+      </c>
+      <c r="C28" s="7" t="s">
         <v>131</v>
-      </c>
-      <c r="B28" s="6" t="s">
-        <v>127</v>
-      </c>
-      <c r="C28" s="7" t="s">
-        <v>132</v>
       </c>
       <c r="D28" s="8" t="s">
         <v>36</v>
@@ -2059,7 +2059,7 @@
         <v>19</v>
       </c>
       <c r="G28" s="7" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="H28" s="6" t="s">
         <v>21</v>
@@ -2074,18 +2074,18 @@
         <v>24</v>
       </c>
       <c r="L28" s="7" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="29" ht="60" customHeight="1" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A29" s="6" t="s">
+        <v>133</v>
+      </c>
+      <c r="B29" s="6" t="s">
+        <v>126</v>
+      </c>
+      <c r="C29" s="7" t="s">
         <v>134</v>
-      </c>
-      <c r="B29" s="6" t="s">
-        <v>127</v>
-      </c>
-      <c r="C29" s="7" t="s">
-        <v>135</v>
       </c>
       <c r="D29" s="8" t="s">
         <v>17</v>
@@ -2097,7 +2097,7 @@
         <v>83</v>
       </c>
       <c r="G29" s="7" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="H29" s="6" t="s">
         <v>21</v>
@@ -2106,24 +2106,24 @@
         <v>32</v>
       </c>
       <c r="J29" s="6" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="K29" s="6" t="s">
         <v>24</v>
       </c>
       <c r="L29" s="7" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="30" ht="60" customHeight="1" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A30" s="6" t="s">
+        <v>137</v>
+      </c>
+      <c r="B30" s="6" t="s">
+        <v>126</v>
+      </c>
+      <c r="C30" s="7" t="s">
         <v>138</v>
-      </c>
-      <c r="B30" s="6" t="s">
-        <v>127</v>
-      </c>
-      <c r="C30" s="7" t="s">
-        <v>139</v>
       </c>
       <c r="D30" s="8" t="s">
         <v>36</v>
@@ -2135,7 +2135,7 @@
         <v>83</v>
       </c>
       <c r="G30" s="7" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="H30" s="6" t="s">
         <v>21</v>
@@ -2150,18 +2150,18 @@
         <v>24</v>
       </c>
       <c r="L30" s="7" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
     </row>
     <row r="31" ht="60" customHeight="1" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A31" s="6" t="s">
+        <v>140</v>
+      </c>
+      <c r="B31" s="6" t="s">
         <v>141</v>
       </c>
-      <c r="B31" s="6" t="s">
+      <c r="C31" s="7" t="s">
         <v>142</v>
-      </c>
-      <c r="C31" s="7" t="s">
-        <v>143</v>
       </c>
       <c r="D31" s="8" t="s">
         <v>17</v>
@@ -2173,7 +2173,7 @@
         <v>19</v>
       </c>
       <c r="G31" s="7" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="H31" s="6" t="s">
         <v>21</v>
@@ -2188,18 +2188,18 @@
         <v>24</v>
       </c>
       <c r="L31" s="7" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
     </row>
     <row r="32" ht="60" customHeight="1" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A32" s="6" t="s">
+        <v>145</v>
+      </c>
+      <c r="B32" s="6" t="s">
+        <v>141</v>
+      </c>
+      <c r="C32" s="7" t="s">
         <v>146</v>
-      </c>
-      <c r="B32" s="6" t="s">
-        <v>142</v>
-      </c>
-      <c r="C32" s="7" t="s">
-        <v>147</v>
       </c>
       <c r="D32" s="8" t="s">
         <v>36</v>
@@ -2211,33 +2211,33 @@
         <v>19</v>
       </c>
       <c r="G32" s="7" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="H32" s="6" t="s">
         <v>21</v>
       </c>
       <c r="I32" s="6" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="J32" s="6" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="K32" s="6" t="s">
         <v>24</v>
       </c>
       <c r="L32" s="7" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
     </row>
     <row r="33" ht="60" customHeight="1" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A33" s="6" t="s">
+        <v>148</v>
+      </c>
+      <c r="B33" s="6" t="s">
         <v>149</v>
       </c>
-      <c r="B33" s="6" t="s">
+      <c r="C33" s="7" t="s">
         <v>150</v>
-      </c>
-      <c r="C33" s="7" t="s">
-        <v>151</v>
       </c>
       <c r="D33" s="8" t="s">
         <v>17</v>
@@ -2249,7 +2249,7 @@
         <v>43</v>
       </c>
       <c r="G33" s="7" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="H33" s="6" t="s">
         <v>21</v>
@@ -2258,27 +2258,27 @@
         <v>74</v>
       </c>
       <c r="J33" s="6" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="K33" s="6" t="s">
         <v>24</v>
       </c>
       <c r="L33" s="7" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="34" ht="60" customHeight="1" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A34" s="6" t="s">
+        <v>153</v>
+      </c>
+      <c r="B34" s="6" t="s">
         <v>154</v>
       </c>
-      <c r="B34" s="6" t="s">
+      <c r="C34" s="7" t="s">
         <v>155</v>
       </c>
-      <c r="C34" s="7" t="s">
+      <c r="D34" s="8" t="s">
         <v>156</v>
-      </c>
-      <c r="D34" s="8" t="s">
-        <v>157</v>
       </c>
       <c r="E34" s="6" t="s">
         <v>88</v>
@@ -2287,7 +2287,7 @@
         <v>19</v>
       </c>
       <c r="G34" s="7" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="H34" s="6" t="s">
         <v>89</v>
@@ -2296,27 +2296,27 @@
         <v>74</v>
       </c>
       <c r="J34" s="6" t="s">
+        <v>158</v>
+      </c>
+      <c r="K34" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="L34" s="7" t="s">
         <v>159</v>
-      </c>
-      <c r="K34" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="L34" s="7" t="s">
-        <v>160</v>
       </c>
     </row>
     <row r="35" ht="60" customHeight="1" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A35" s="6" t="s">
+        <v>160</v>
+      </c>
+      <c r="B35" s="6" t="s">
+        <v>154</v>
+      </c>
+      <c r="C35" s="7" t="s">
         <v>161</v>
       </c>
-      <c r="B35" s="6" t="s">
-        <v>155</v>
-      </c>
-      <c r="C35" s="7" t="s">
-        <v>162</v>
-      </c>
       <c r="D35" s="8" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="E35" s="6" t="s">
         <v>29</v>
@@ -2325,7 +2325,7 @@
         <v>43</v>
       </c>
       <c r="G35" s="7" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="H35" s="6" t="s">
         <v>31</v>
@@ -2334,27 +2334,27 @@
         <v>74</v>
       </c>
       <c r="J35" s="6" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="K35" s="6" t="s">
         <v>24</v>
       </c>
       <c r="L35" s="7" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="36" ht="60" customHeight="1" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A36" s="6" t="s">
+        <v>164</v>
+      </c>
+      <c r="B36" s="6" t="s">
+        <v>154</v>
+      </c>
+      <c r="C36" s="7" t="s">
         <v>165</v>
       </c>
-      <c r="B36" s="6" t="s">
-        <v>155</v>
-      </c>
-      <c r="C36" s="7" t="s">
-        <v>166</v>
-      </c>
       <c r="D36" s="8" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="E36" s="6" t="s">
         <v>88</v>
@@ -2363,36 +2363,36 @@
         <v>43</v>
       </c>
       <c r="G36" s="7" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="H36" s="6" t="s">
         <v>89</v>
       </c>
       <c r="I36" s="6" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="J36" s="6" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="K36" s="6" t="s">
-        <v>90</v>
+        <v>24</v>
       </c>
       <c r="L36" s="7" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="37" ht="60" customHeight="1" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A37" s="6" t="s">
+        <v>168</v>
+      </c>
+      <c r="B37" s="6" t="s">
         <v>169</v>
       </c>
-      <c r="B37" s="6" t="s">
+      <c r="C37" s="7" t="s">
         <v>170</v>
       </c>
-      <c r="C37" s="7" t="s">
+      <c r="D37" s="8" t="s">
         <v>171</v>
-      </c>
-      <c r="D37" s="8" t="s">
-        <v>172</v>
       </c>
       <c r="E37" s="6" t="s">
         <v>18</v>
@@ -2401,7 +2401,7 @@
         <v>43</v>
       </c>
       <c r="G37" s="7" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="H37" s="6" t="s">
         <v>21</v>
@@ -2410,24 +2410,24 @@
         <v>74</v>
       </c>
       <c r="J37" s="6" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="K37" s="6" t="s">
         <v>24</v>
       </c>
       <c r="L37" s="7" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
     </row>
     <row r="38" ht="60" customHeight="1" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A38" s="6" t="s">
+        <v>173</v>
+      </c>
+      <c r="B38" s="6" t="s">
+        <v>169</v>
+      </c>
+      <c r="C38" s="7" t="s">
         <v>174</v>
-      </c>
-      <c r="B38" s="6" t="s">
-        <v>170</v>
-      </c>
-      <c r="C38" s="7" t="s">
-        <v>175</v>
       </c>
       <c r="D38" s="8" t="s">
         <v>17</v>
@@ -2439,7 +2439,7 @@
         <v>19</v>
       </c>
       <c r="G38" s="7" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="H38" s="6" t="s">
         <v>21</v>
@@ -2448,27 +2448,27 @@
         <v>57</v>
       </c>
       <c r="J38" s="6" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="K38" s="6" t="s">
         <v>24</v>
       </c>
       <c r="L38" s="7" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
     </row>
     <row r="39" ht="60" customHeight="1" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A39" s="6" t="s">
+        <v>176</v>
+      </c>
+      <c r="B39" s="6" t="s">
+        <v>169</v>
+      </c>
+      <c r="C39" s="7" t="s">
         <v>177</v>
       </c>
-      <c r="B39" s="6" t="s">
-        <v>170</v>
-      </c>
-      <c r="C39" s="7" t="s">
-        <v>178</v>
-      </c>
       <c r="D39" s="8" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="E39" s="6" t="s">
         <v>18</v>
@@ -2477,22 +2477,22 @@
         <v>43</v>
       </c>
       <c r="G39" s="7" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="H39" s="6" t="s">
         <v>21</v>
       </c>
       <c r="I39" s="6" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="J39" s="6" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="K39" s="6" t="s">
+        <v>178</v>
+      </c>
+      <c r="L39" s="7" t="s">
         <v>179</v>
-      </c>
-      <c r="L39" s="7" t="s">
-        <v>180</v>
       </c>
     </row>
   </sheetData>
@@ -2541,24 +2541,24 @@
   <sheetData>
     <row r="1" ht="16.5" customHeight="1" spans="1:1" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="9" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
     </row>
     <row r="3" ht="13.5" customHeight="1" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="10" t="s">
+        <v>181</v>
+      </c>
+      <c r="B3" s="10" t="s">
         <v>182</v>
       </c>
-      <c r="B3" s="10" t="s">
+      <c r="C3" s="10" t="s">
         <v>183</v>
       </c>
-      <c r="C3" s="10" t="s">
+      <c r="D3" s="10" t="s">
         <v>184</v>
       </c>
-      <c r="D3" s="10" t="s">
-        <v>90</v>
-      </c>
       <c r="E3" s="10" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="F3" s="10" t="s">
         <v>24</v>
@@ -2579,21 +2579,27 @@
       </c>
       <c r="C4" s="11">
         <f>COUNTIF('Task Sprint 4'!$E$5:$E$39,A4)</f>
+        <v>0</v>
       </c>
       <c r="D4" s="11">
         <f>COUNTIFS('Task Sprint 4'!$E$5:$E$39,$A4,'Task Sprint 4'!$K$5:$K$39,"To Do")</f>
+        <v>0</v>
       </c>
       <c r="E4" s="11">
         <f>COUNTIFS('Task Sprint 4'!$E$5:$E$39,$A4,'Task Sprint 4'!$K$5:$K$39,"In Progress")</f>
+        <v>0</v>
       </c>
       <c r="F4" s="11">
         <f>COUNTIFS('Task Sprint 4'!$E$5:$E$39,$A4,'Task Sprint 4'!$K$5:$K$39,"Review")</f>
+        <v>0</v>
       </c>
       <c r="G4" s="11">
         <f>COUNTIFS('Task Sprint 4'!$E$5:$E$39,$A4,'Task Sprint 4'!$K$5:$K$39,"Done")</f>
+        <v>0</v>
       </c>
       <c r="H4" s="12">
         <f>IF(C4=0,0,G4/C4)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="5" ht="13.5" customHeight="1" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -2605,21 +2611,27 @@
       </c>
       <c r="C5" s="11">
         <f>COUNTIF('Task Sprint 4'!$E$5:$E$39,A5)</f>
+        <v>17</v>
       </c>
       <c r="D5" s="11">
         <f>COUNTIFS('Task Sprint 4'!$E$5:$E$39,$A5,'Task Sprint 4'!$K$5:$K$39,"To Do")</f>
+        <v>0</v>
       </c>
       <c r="E5" s="11">
         <f>COUNTIFS('Task Sprint 4'!$E$5:$E$39,$A5,'Task Sprint 4'!$K$5:$K$39,"In Progress")</f>
+        <v>1</v>
       </c>
       <c r="F5" s="11">
         <f>COUNTIFS('Task Sprint 4'!$E$5:$E$39,$A5,'Task Sprint 4'!$K$5:$K$39,"Review")</f>
+        <v>16</v>
       </c>
       <c r="G5" s="11">
         <f>COUNTIFS('Task Sprint 4'!$E$5:$E$39,$A5,'Task Sprint 4'!$K$5:$K$39,"Done")</f>
+        <v>0</v>
       </c>
       <c r="H5" s="12">
         <f>IF(C5=0,0,G5/C5)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="6" ht="13.5" customHeight="1" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -2631,21 +2643,27 @@
       </c>
       <c r="C6" s="11">
         <f>COUNTIF('Task Sprint 4'!$E$5:$E$39,A6)</f>
+        <v>11</v>
       </c>
       <c r="D6" s="11">
         <f>COUNTIFS('Task Sprint 4'!$E$5:$E$39,$A6,'Task Sprint 4'!$K$5:$K$39,"To Do")</f>
+        <v>0</v>
       </c>
       <c r="E6" s="11">
         <f>COUNTIFS('Task Sprint 4'!$E$5:$E$39,$A6,'Task Sprint 4'!$K$5:$K$39,"In Progress")</f>
+        <v>0</v>
       </c>
       <c r="F6" s="11">
         <f>COUNTIFS('Task Sprint 4'!$E$5:$E$39,$A6,'Task Sprint 4'!$K$5:$K$39,"Review")</f>
+        <v>11</v>
       </c>
       <c r="G6" s="11">
         <f>COUNTIFS('Task Sprint 4'!$E$5:$E$39,$A6,'Task Sprint 4'!$K$5:$K$39,"Done")</f>
+        <v>0</v>
       </c>
       <c r="H6" s="12">
         <f>IF(C6=0,0,G6/C6)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="7" ht="13.5" customHeight="1" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -2657,21 +2675,27 @@
       </c>
       <c r="C7" s="11">
         <f>COUNTIF('Task Sprint 4'!$E$5:$E$39,A7)</f>
+        <v>7</v>
       </c>
       <c r="D7" s="11">
         <f>COUNTIFS('Task Sprint 4'!$E$5:$E$39,$A7,'Task Sprint 4'!$K$5:$K$39,"To Do")</f>
+        <v>0</v>
       </c>
       <c r="E7" s="11">
         <f>COUNTIFS('Task Sprint 4'!$E$5:$E$39,$A7,'Task Sprint 4'!$K$5:$K$39,"In Progress")</f>
+        <v>0</v>
       </c>
       <c r="F7" s="11">
         <f>COUNTIFS('Task Sprint 4'!$E$5:$E$39,$A7,'Task Sprint 4'!$K$5:$K$39,"Review")</f>
+        <v>7</v>
       </c>
       <c r="G7" s="11">
         <f>COUNTIFS('Task Sprint 4'!$E$5:$E$39,$A7,'Task Sprint 4'!$K$5:$K$39,"Done")</f>
+        <v>0</v>
       </c>
       <c r="H7" s="12">
         <f>IF(C7=0,0,G7/C7)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="8" ht="13.5" customHeight="1" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -2680,21 +2704,27 @@
       </c>
       <c r="C8" s="1">
         <f>SUM(C4:C7)</f>
+        <v>NaN</v>
       </c>
       <c r="D8" s="1">
         <f>SUM(D4:D7)</f>
+        <v>NaN</v>
       </c>
       <c r="E8" s="1">
         <f>SUM(E4:E7)</f>
+        <v>NaN</v>
       </c>
       <c r="F8" s="1">
         <f>SUM(F4:F7)</f>
+        <v>NaN</v>
       </c>
       <c r="G8" s="1">
         <f>SUM(G4:G7)</f>
+        <v>NaN</v>
       </c>
       <c r="H8" s="14">
         <f>IF(C8=0,0,G8/C8)</f>
+        <v>NaN</v>
       </c>
     </row>
     <row r="10" ht="13.5" customHeight="1" spans="1:1" s="2" customFormat="1" x14ac:dyDescent="0.25">

</xml_diff>